<commit_message>
Synchronise les données Shopify avec le dataset validé
Aligne commandes, NPS et coûts produits sur la bible de données
harmonisée utilisée pour les moteurs Avant-vente et Impact & confiance.
Rétablit sur le dépôt les données ayant servi aux rejeux fonctionnels
et à la validation portfolio. Aucun code ni seuil métier modifié.
</commit_message>
<xml_diff>
--- a/data_shopify/product_costs_fictif.xlsx
+++ b/data_shopify/product_costs_fictif.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -842,6 +842,38 @@
         <v>0</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ETR-RCH-001</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Recharge</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Étreinte</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>42</v>
+      </c>
+      <c r="E14" t="n">
+        <v>35</v>
+      </c>
+      <c r="F14" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="G14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>